<commit_message>
variable of interest is created in terms of Budget Balance = T - G --> re converted the labelling script, but need to focus and think about the interpretation of the results, I have some doubts
</commit_message>
<xml_diff>
--- a/FISCAL/Fiscal_LDC/1_Classified_Fiscal_Events_Top5Percent.xlsx
+++ b/FISCAL/Fiscal_LDC/1_Classified_Fiscal_Events_Top5Percent.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lorenzodelcol/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lorenzodelcol/Desktop/GIT/RA_4_Caggiano/FISCAL/Fiscal_LDC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8B87C24-8E4E-3647-A767-03BCDD38F5D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F03E5694-8420-6740-AF68-53AD373A6028}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="124">
   <si>
     <t>date</t>
   </si>
@@ -70,15 +70,9 @@
     <t>1993-02-15</t>
   </si>
   <si>
-    <t>The massive fiscal shock on 1993-02-15 was primarily driven by the widely reported and leaked details of President Clinton's comprehensive economic plan, which was formally unveiled on February 17, 1993. In the 48-to-72-hour window around this date, news outlets extensively covered the plan's components, with a significant focus on proposed tax increases. These included raising the top marginal income tax rates for individuals and corporations, increasing the taxation of Social Security benefits for higher earners, and introducing a new energy (BTU) tax. While the plan also included spending cuts, the substantial and broad-reaching tax increases were a dominant and highly discussed feature, likely triggering the outsized macroeconomic reaction.</t>
-  </si>
-  <si>
     <t>1993-08-09</t>
   </si>
   <si>
-    <t>The massive fiscal shock on 1993-08-09 is primarily driven by the final legislative actions surrounding the Omnibus Budget Reconciliation Act of 1993 (OBRA-93). The bill passed the House on August 5th and the Senate on August 6th, and was signed into law by President Clinton on August 10th. While OBRA-93 was a comprehensive deficit reduction package that included both significant tax increases and spending cuts, the spending reductions, totaling approximately $255 billion over five years (including cuts to Medicare, defense, and other discretionary programs), were slightly larger in magnitude than the tax increases ($241 billion). Therefore, Government Spending (G) is identified as the dominant factor.</t>
-  </si>
-  <si>
     <t>1995-10-20</t>
   </si>
   <si>
@@ -371,9 +365,6 @@
   </si>
   <si>
     <t>Lorenzo</t>
-  </si>
-  <si>
-    <t>Sbagliato, questo dovrebbe essere o un G negative (G cuts) o un Tax Positive (tax increase) --&gt; LLM correttamente fa fatica ad identificarlo, è uno shock che comprende sia T che G, ma visto che G cut è leggermente maggiore di Tax incrase lo identifica come un Positive G --&gt; mentre io penso sia un Positive T se dobbiamo classificarlo tra G e T per forza. --&gt; però forzare l'identificazione può portare ad avere measurement error se po questi shock vengono usati in Proxy SVAR of LP</t>
   </si>
   <si>
     <r>
@@ -486,12 +477,137 @@
       <t xml:space="preserve"> supply-side economic philosophy and represented a massive, defining shift in fiscal policy, making them the most dominant factor in the macroeconomic news cycle and the primary driver of the fiscal shock on this date.</t>
     </r>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The massive fiscal shock on 1993-02-15 was primarily driven by the widely reported and leaked details of President Clinton's comprehensive economic plan, which was formally unveiled on February 17, 1993. In the 48-to-72-hour window around this date, news outlets extensively covered the plan's components, with a significant </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri (Corpo)"/>
+      </rPr>
+      <t>focus on proposed tax increases</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri (Corpo)"/>
+      </rPr>
+      <t>These included raising the top marginal income tax rates for individuals and corporations, increasing the taxation of Social Security benefits for higher earners</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, and introducing a new energy (BTU) tax. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri (Corpo)"/>
+      </rPr>
+      <t>While the plan also included spending cuts, the substantial and broad-reaching tax increases</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> were a dominant and highly discussed feature, likely triggering the outsized macroeconomic reaction.</t>
+    </r>
+  </si>
+  <si>
+    <t>corretto</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The massive fiscal shock on 1993-08-09 is primarily driven by the final legislative actions surrounding the Omnibus Budget Reconciliation Act of 1993 (OBRA-93). The bill passed the House on August 5th and the Senate on August 6th, and was signed into law by President Clinton on August 10th. While </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri (Corpo)"/>
+      </rPr>
+      <t xml:space="preserve">OBRA-93 was a comprehensive deficit reduction package that included both significant tax increases and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri (Corpo)"/>
+      </rPr>
+      <t>spending cuts</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri (Corpo)"/>
+      </rPr>
+      <t>the spending reductions, totaling approximately $255 billion over five years (including cuts to Medicare, defense, and other discretionary programs), were slightly larger in magnitude than the tax increases ($241 billion)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri (Corpo)"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Therefore, Government Spending (G) is identified as the dominant factor.</t>
+    </r>
+  </si>
+  <si>
+    <t>Questo dovrebbe essere o un G negative (G cuts) o un Tax Positive (tax increase) --&gt; Dal riassunto del LLM non vengono citati numeri per Tax Increases, però vengono specificare esattamente G Cuts, la somma è 496 billio cuts in 5 years, quindi nel valore attuale è minore, e viene riflesso nel 415 del pv change--&gt; Però questo dovrebbe essere un G cut, quindi Negative G --&gt; Anche qui il problema sembra essere alla fonte, dovrebbe avere segno opposto</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -513,6 +629,20 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri (Corpo)"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -933,7 +1063,7 @@
         <v>9</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="48" x14ac:dyDescent="0.2">
@@ -952,6 +1082,9 @@
       <c r="J2" s="3" t="s">
         <v>11</v>
       </c>
+      <c r="K2" s="3" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="3" spans="1:11" ht="80" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -970,7 +1103,10 @@
         <v>3</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>118</v>
+        <v>115</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="64" x14ac:dyDescent="0.2">
@@ -990,10 +1126,10 @@
         <v>3</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="112" x14ac:dyDescent="0.2">
@@ -1013,10 +1149,10 @@
         <v>3</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="96" x14ac:dyDescent="0.2">
@@ -1036,12 +1172,15 @@
         <v>3</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>16</v>
+        <v>120</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="7" spans="1:11" s="4" customFormat="1" ht="96" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" s="4">
         <v>415.00617525975582</v>
@@ -1056,15 +1195,15 @@
         <v>2</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>18</v>
+        <v>122</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="80" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B8">
         <v>87.86865544914879</v>
@@ -1079,12 +1218,12 @@
         <v>2</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="80" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B9">
         <v>503.95253613149163</v>
@@ -1099,12 +1238,12 @@
         <v>2</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:11" s="4" customFormat="1" ht="96" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B10" s="4">
         <v>269.90349136839302</v>
@@ -1119,13 +1258,13 @@
         <v>3</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="K10" s="5"/>
     </row>
     <row r="11" spans="1:11" ht="80" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B11">
         <v>96.113815876822159</v>
@@ -1140,12 +1279,12 @@
         <v>2</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="80" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B12">
         <v>-151.4124688981552</v>
@@ -1160,12 +1299,12 @@
         <v>3</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B13">
         <v>-189.26896537445259</v>
@@ -1180,12 +1319,12 @@
         <v>2</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="80" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B14">
         <v>-202.9847143898794</v>
@@ -1200,12 +1339,12 @@
         <v>2</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:11" s="4" customFormat="1" ht="96" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B15" s="4">
         <v>-156.82028933312361</v>
@@ -1220,13 +1359,13 @@
         <v>3</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="K15" s="5"/>
     </row>
     <row r="16" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B16">
         <v>-111.53031497214729</v>
@@ -1241,12 +1380,12 @@
         <v>2</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17" spans="1:11" s="4" customFormat="1" ht="64" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B17" s="4">
         <v>-232.4417007363582</v>
@@ -1261,13 +1400,13 @@
         <v>3</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="K17" s="5"/>
     </row>
     <row r="18" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B18">
         <v>-249.5974496202042</v>
@@ -1282,12 +1421,12 @@
         <v>3</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B19">
         <v>-529.17092465149221</v>
@@ -1302,12 +1441,12 @@
         <v>3</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="80" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B20">
         <v>-146.78116308087399</v>
@@ -1322,12 +1461,12 @@
         <v>3</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21" spans="1:11" s="4" customFormat="1" ht="64" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B21" s="4">
         <v>-148.2249838679231</v>
@@ -1342,13 +1481,13 @@
         <v>2</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="K21" s="5"/>
     </row>
     <row r="22" spans="1:11" s="4" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B22" s="4">
         <v>-246.37821805298611</v>
@@ -1363,734 +1502,734 @@
         <v>2</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="K22" s="5"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B23">
         <v>-87.722760721289646</v>
       </c>
       <c r="I23" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B24">
         <v>-172.83179207606861</v>
       </c>
       <c r="I24" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B25">
         <v>-141.21637310006321</v>
       </c>
       <c r="I25" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B26">
         <v>-161.06960258571269</v>
       </c>
       <c r="I26" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B27">
         <v>-202.57199864455171</v>
       </c>
       <c r="I27" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B28">
         <v>-163.31804264167221</v>
       </c>
       <c r="I28" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B29">
         <v>-152.92923732444689</v>
       </c>
       <c r="I29" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B30">
         <v>-248.45256107553939</v>
       </c>
       <c r="I30" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B31">
         <v>-1199.209304600121</v>
       </c>
       <c r="I31" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B32">
         <v>391.86138027946919</v>
       </c>
       <c r="I32" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B33">
         <v>108.2317293907218</v>
       </c>
       <c r="I33" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B34">
         <v>-261.5619937281686</v>
       </c>
       <c r="I34" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B35">
         <v>-107.88515860470319</v>
       </c>
       <c r="I35" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B36">
         <v>-182.8788031923161</v>
       </c>
       <c r="I36" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B37">
         <v>-183.42798776198691</v>
       </c>
       <c r="I37" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B38">
         <v>-192.6147477522621</v>
       </c>
       <c r="I38" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B39">
         <v>1748.3550672281619</v>
       </c>
       <c r="I39" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B40">
         <v>-402.29826229755741</v>
       </c>
       <c r="I40" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B41">
         <v>-138.6862505995087</v>
       </c>
       <c r="I41" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B42">
         <v>-230.6493234163718</v>
       </c>
       <c r="I42" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B43">
         <v>-1782.0190466026061</v>
       </c>
       <c r="I43" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B44">
         <v>92.217497605615179</v>
       </c>
       <c r="I44" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B45">
         <v>477.6407083384322</v>
       </c>
       <c r="I45" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B46">
         <v>161.86215832132129</v>
       </c>
       <c r="I46" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B47">
         <v>-273.05665714327893</v>
       </c>
       <c r="I47" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B48">
         <v>146.1973513648887</v>
       </c>
       <c r="I48" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B49">
         <v>114.64160770773699</v>
       </c>
       <c r="I49" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B50">
         <v>133.22528008284601</v>
       </c>
       <c r="I50" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B51">
         <v>-203.91844288041531</v>
       </c>
       <c r="I51" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B52">
         <v>-446.16251606515442</v>
       </c>
       <c r="I52" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B53">
         <v>93.513879965796519</v>
       </c>
       <c r="I53" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B54">
         <v>-192.33581616385399</v>
       </c>
       <c r="I54" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B55">
         <v>-176.92371282897821</v>
       </c>
       <c r="I55" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B56">
         <v>-207.28690503464159</v>
       </c>
       <c r="I56" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B57">
         <v>-165.0011653349533</v>
       </c>
       <c r="I57" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B58">
         <v>-276.38945753885929</v>
       </c>
       <c r="I58" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B59">
         <v>-120.1009540721557</v>
       </c>
       <c r="I59" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B60">
         <v>-143.1113566126474</v>
       </c>
       <c r="I60" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B61">
         <v>-428.79182457489537</v>
       </c>
       <c r="I61" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B62">
         <v>-657.44251936497039</v>
       </c>
       <c r="I62" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B63">
         <v>-2041.780924862881</v>
       </c>
       <c r="I63" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B64">
         <v>615.86628034078262</v>
       </c>
       <c r="I64" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B65">
         <v>-169.59377942450891</v>
       </c>
       <c r="I65" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B66">
         <v>-89.290345938567185</v>
       </c>
       <c r="I66" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B67">
         <v>-984.66883793782119</v>
       </c>
       <c r="I67" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B68">
         <v>-476.00040837070628</v>
       </c>
       <c r="I68" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B69">
         <v>179.54472327198059</v>
       </c>
       <c r="I69" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B70">
         <v>166.5617790268318</v>
       </c>
       <c r="I70" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B71">
         <v>-180.10847121243651</v>
       </c>
       <c r="I71" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B72">
         <v>-179.83145417219279</v>
       </c>
       <c r="I72" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B73">
         <v>-552.22911894411504</v>
       </c>
       <c r="I73" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B74">
         <v>-234.61385357430859</v>
       </c>
       <c r="I74" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B75">
         <v>202.46136313468651</v>
       </c>
       <c r="I75" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B76">
         <v>-106.5970450688274</v>
       </c>
       <c r="I76" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B77">
         <v>-1051.6635574296449</v>
       </c>
       <c r="I77" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B78">
         <v>-540.46550103801428</v>
       </c>
       <c r="I78" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B79">
         <v>-197.7441439976659</v>
       </c>
       <c r="I79" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B80">
         <v>-700.94624941174834</v>
       </c>
       <c r="I80" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B81">
         <v>-412.80577790767512</v>
       </c>
       <c r="I81" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B82">
         <v>-640.16266533291071</v>
       </c>
       <c r="I82" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B83">
         <v>-515.37490113762385</v>
       </c>
       <c r="I83" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B84">
         <v>-214.08815960384689</v>
       </c>
       <c r="I84" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B85">
         <v>844.14424346889075</v>
       </c>
       <c r="I85" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B86">
         <v>-377.90035722856311</v>
       </c>
       <c r="I86" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B87">
         <v>-200.3390287029126</v>
       </c>
       <c r="I87" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B88">
         <v>-236.26023728124079</v>
       </c>
       <c r="I88" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
still the result of the prompt is not good
</commit_message>
<xml_diff>
--- a/FISCAL/Fiscal_LDC/1_Classified_Fiscal_Events_Top5Percent.xlsx
+++ b/FISCAL/Fiscal_LDC/1_Classified_Fiscal_Events_Top5Percent.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lorenzodelcol/Desktop/GIT/RA_4_Caggiano/FISCAL/Fiscal_LDC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F03E5694-8420-6740-AF68-53AD373A6028}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B4C8285-C15C-CC40-B2C7-0D7E6C0999CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20320" yWindow="600" windowWidth="20320" windowHeight="14320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -100,9 +100,6 @@
     <t>2001-01-26</t>
   </si>
   <si>
-    <t>The period immediately following President George W. Bush's inauguration (January 20, 2001) was dominated by his administration's aggressive push for a significant tax cut package. Around January 26, 2001, news cycles were heavily focused on Bush's meetings with congressional leaders and public statements advocating for his proposed tax cuts, leveraging the projected budget surplus. This marked the beginning of the legislative effort that would eventually lead to the Economic Growth and Tax Relief Reconciliation Act of 2001 (EGTRRA), representing a major shift in tax policy and a significant fiscal shock.</t>
-  </si>
-  <si>
     <t>2001-09-12</t>
   </si>
   <si>
@@ -601,6 +598,39 @@
   </si>
   <si>
     <t>Questo dovrebbe essere o un G negative (G cuts) o un Tax Positive (tax increase) --&gt; Dal riassunto del LLM non vengono citati numeri per Tax Increases, però vengono specificare esattamente G Cuts, la somma è 496 billio cuts in 5 years, quindi nel valore attuale è minore, e viene riflesso nel 415 del pv change--&gt; Però questo dovrebbe essere un G cut, quindi Negative G --&gt; Anche qui il problema sembra essere alla fonte, dovrebbe avere segno opposto</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The period immediately following President George W. Bush's inauguration (January 20, 2001) was dominated by his administration's aggressive push for a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri (Corpo)"/>
+      </rPr>
+      <t>significant tax cut packag</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>e</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Around January 26, 2001, news cycles were heavily focused on Bush's meetings with congressional leaders and public statements advocating for his proposed tax cuts, leveraging the projected budget surplus. This marked the beginning of the legislative effort that would eventually lead to the Economic Growth and Tax Relief Reconciliation Act of 2001 (EGTRRA), representing a major shift in tax policy and a significant fiscal shock.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1063,7 +1093,7 @@
         <v>9</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="48" x14ac:dyDescent="0.2">
@@ -1083,7 +1113,7 @@
         <v>11</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="80" x14ac:dyDescent="0.2">
@@ -1103,10 +1133,10 @@
         <v>3</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="64" x14ac:dyDescent="0.2">
@@ -1126,10 +1156,10 @@
         <v>3</v>
       </c>
       <c r="J4" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="K4" s="3" t="s">
         <v>117</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="112" x14ac:dyDescent="0.2">
@@ -1149,10 +1179,10 @@
         <v>3</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="96" x14ac:dyDescent="0.2">
@@ -1172,10 +1202,10 @@
         <v>3</v>
       </c>
       <c r="J6" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="K6" s="3" t="s">
         <v>120</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="7" spans="1:11" s="4" customFormat="1" ht="96" x14ac:dyDescent="0.2">
@@ -1195,10 +1225,10 @@
         <v>2</v>
       </c>
       <c r="J7" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="K7" s="5" t="s">
         <v>122</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="80" x14ac:dyDescent="0.2">
@@ -1299,12 +1329,12 @@
         <v>3</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>26</v>
+        <v>123</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B13">
         <v>-189.26896537445259</v>
@@ -1319,12 +1349,12 @@
         <v>2</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="80" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B14">
         <v>-202.9847143898794</v>
@@ -1339,12 +1369,12 @@
         <v>2</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:11" s="4" customFormat="1" ht="96" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B15" s="4">
         <v>-156.82028933312361</v>
@@ -1359,13 +1389,13 @@
         <v>3</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="K15" s="5"/>
     </row>
     <row r="16" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B16">
         <v>-111.53031497214729</v>
@@ -1380,12 +1410,12 @@
         <v>2</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:11" s="4" customFormat="1" ht="64" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B17" s="4">
         <v>-232.4417007363582</v>
@@ -1400,13 +1430,13 @@
         <v>3</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K17" s="5"/>
     </row>
     <row r="18" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B18">
         <v>-249.5974496202042</v>
@@ -1421,12 +1451,12 @@
         <v>3</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B19">
         <v>-529.17092465149221</v>
@@ -1441,12 +1471,12 @@
         <v>3</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="80" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B20">
         <v>-146.78116308087399</v>
@@ -1461,12 +1491,12 @@
         <v>3</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:11" s="4" customFormat="1" ht="64" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B21" s="4">
         <v>-148.2249838679231</v>
@@ -1481,13 +1511,13 @@
         <v>2</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K21" s="5"/>
     </row>
     <row r="22" spans="1:11" s="4" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B22" s="4">
         <v>-246.37821805298611</v>
@@ -1502,734 +1532,734 @@
         <v>2</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="K22" s="5"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B23">
         <v>-87.722760721289646</v>
       </c>
       <c r="I23" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B24">
         <v>-172.83179207606861</v>
       </c>
       <c r="I24" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B25">
         <v>-141.21637310006321</v>
       </c>
       <c r="I25" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B26">
         <v>-161.06960258571269</v>
       </c>
       <c r="I26" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B27">
         <v>-202.57199864455171</v>
       </c>
       <c r="I27" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B28">
         <v>-163.31804264167221</v>
       </c>
       <c r="I28" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B29">
         <v>-152.92923732444689</v>
       </c>
       <c r="I29" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B30">
         <v>-248.45256107553939</v>
       </c>
       <c r="I30" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B31">
         <v>-1199.209304600121</v>
       </c>
       <c r="I31" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B32">
         <v>391.86138027946919</v>
       </c>
       <c r="I32" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B33">
         <v>108.2317293907218</v>
       </c>
       <c r="I33" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B34">
         <v>-261.5619937281686</v>
       </c>
       <c r="I34" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B35">
         <v>-107.88515860470319</v>
       </c>
       <c r="I35" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B36">
         <v>-182.8788031923161</v>
       </c>
       <c r="I36" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B37">
         <v>-183.42798776198691</v>
       </c>
       <c r="I37" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B38">
         <v>-192.6147477522621</v>
       </c>
       <c r="I38" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B39">
         <v>1748.3550672281619</v>
       </c>
       <c r="I39" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B40">
         <v>-402.29826229755741</v>
       </c>
       <c r="I40" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B41">
         <v>-138.6862505995087</v>
       </c>
       <c r="I41" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B42">
         <v>-230.6493234163718</v>
       </c>
       <c r="I42" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B43">
         <v>-1782.0190466026061</v>
       </c>
       <c r="I43" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B44">
         <v>92.217497605615179</v>
       </c>
       <c r="I44" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B45">
         <v>477.6407083384322</v>
       </c>
       <c r="I45" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B46">
         <v>161.86215832132129</v>
       </c>
       <c r="I46" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B47">
         <v>-273.05665714327893</v>
       </c>
       <c r="I47" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B48">
         <v>146.1973513648887</v>
       </c>
       <c r="I48" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B49">
         <v>114.64160770773699</v>
       </c>
       <c r="I49" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B50">
         <v>133.22528008284601</v>
       </c>
       <c r="I50" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B51">
         <v>-203.91844288041531</v>
       </c>
       <c r="I51" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B52">
         <v>-446.16251606515442</v>
       </c>
       <c r="I52" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B53">
         <v>93.513879965796519</v>
       </c>
       <c r="I53" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B54">
         <v>-192.33581616385399</v>
       </c>
       <c r="I54" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B55">
         <v>-176.92371282897821</v>
       </c>
       <c r="I55" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B56">
         <v>-207.28690503464159</v>
       </c>
       <c r="I56" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B57">
         <v>-165.0011653349533</v>
       </c>
       <c r="I57" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B58">
         <v>-276.38945753885929</v>
       </c>
       <c r="I58" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B59">
         <v>-120.1009540721557</v>
       </c>
       <c r="I59" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B60">
         <v>-143.1113566126474</v>
       </c>
       <c r="I60" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B61">
         <v>-428.79182457489537</v>
       </c>
       <c r="I61" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B62">
         <v>-657.44251936497039</v>
       </c>
       <c r="I62" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B63">
         <v>-2041.780924862881</v>
       </c>
       <c r="I63" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B64">
         <v>615.86628034078262</v>
       </c>
       <c r="I64" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B65">
         <v>-169.59377942450891</v>
       </c>
       <c r="I65" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B66">
         <v>-89.290345938567185</v>
       </c>
       <c r="I66" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B67">
         <v>-984.66883793782119</v>
       </c>
       <c r="I67" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B68">
         <v>-476.00040837070628</v>
       </c>
       <c r="I68" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B69">
         <v>179.54472327198059</v>
       </c>
       <c r="I69" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B70">
         <v>166.5617790268318</v>
       </c>
       <c r="I70" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B71">
         <v>-180.10847121243651</v>
       </c>
       <c r="I71" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B72">
         <v>-179.83145417219279</v>
       </c>
       <c r="I72" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B73">
         <v>-552.22911894411504</v>
       </c>
       <c r="I73" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B74">
         <v>-234.61385357430859</v>
       </c>
       <c r="I74" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B75">
         <v>202.46136313468651</v>
       </c>
       <c r="I75" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B76">
         <v>-106.5970450688274</v>
       </c>
       <c r="I76" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B77">
         <v>-1051.6635574296449</v>
       </c>
       <c r="I77" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B78">
         <v>-540.46550103801428</v>
       </c>
       <c r="I78" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B79">
         <v>-197.7441439976659</v>
       </c>
       <c r="I79" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B80">
         <v>-700.94624941174834</v>
       </c>
       <c r="I80" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B81">
         <v>-412.80577790767512</v>
       </c>
       <c r="I81" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B82">
         <v>-640.16266533291071</v>
       </c>
       <c r="I82" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B83">
         <v>-515.37490113762385</v>
       </c>
       <c r="I83" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B84">
         <v>-214.08815960384689</v>
       </c>
       <c r="I84" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B85">
         <v>844.14424346889075</v>
       </c>
       <c r="I85" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B86">
         <v>-377.90035722856311</v>
       </c>
       <c r="I86" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B87">
         <v>-200.3390287029126</v>
       </c>
       <c r="I87" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B88">
         <v>-236.26023728124079</v>
       </c>
       <c r="I88" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>